<commit_message>
Cập nhật file excel deadline
</commit_message>
<xml_diff>
--- a/deadline_laptrinhmang.xlsx
+++ b/deadline_laptrinhmang.xlsx
@@ -1,35 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6F682DD9AFBBD5EA/Tài liệu/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GITHUB\UDM_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C8656E6-9CC3-44DC-9F43-42C2C4FCE7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA6817F-4768-4E4A-85FA-2D069DF3CE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{4996BFC1-5545-47D6-BEAA-54FAD06ABAD6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4996BFC1-5545-47D6-BEAA-54FAD06ABAD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -834,7 +823,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1301,19 +1290,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0401913-6D54-40AB-B28F-C9358A79A9F4}">
   <dimension ref="A1:P65"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="2" max="2" width="15.5703125" customWidth="1"/>
-    <col min="3" max="3" width="30.85546875" customWidth="1"/>
-    <col min="4" max="4" width="30.7109375" customWidth="1"/>
-    <col min="5" max="5" width="67.140625" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="30.6640625" customWidth="1"/>
+    <col min="5" max="5" width="67.109375" customWidth="1"/>
     <col min="6" max="6" width="19" customWidth="1"/>
-    <col min="7" max="7" width="29.5703125" customWidth="1"/>
-    <col min="8" max="8" width="23.85546875" customWidth="1"/>
+    <col min="7" max="7" width="29.5546875" customWidth="1"/>
+    <col min="8" max="8" width="23.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.25" thickBot="1">
+    <row r="1" spans="1:8" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -1339,7 +1328,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="31.5" thickTop="1" thickBot="1">
+    <row r="2" spans="1:8" ht="28.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1365,7 +1354,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="30.75" thickBot="1">
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1391,7 +1380,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1">
+    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1415,7 +1404,7 @@
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1">
+    <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1439,7 +1428,7 @@
       </c>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" ht="15.75" thickBot="1">
+    <row r="6" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1459,11 +1448,11 @@
         <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="15.75" thickBot="1">
+    <row r="7" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1483,11 +1472,11 @@
         <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" ht="15.75" thickBot="1">
+    <row r="8" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1511,7 +1500,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1535,7 +1524,7 @@
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="15.75" thickBot="1">
+    <row r="10" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1559,7 +1548,7 @@
       </c>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" ht="15.75" thickBot="1">
+    <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1583,7 +1572,7 @@
       </c>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" ht="15.75" thickBot="1">
+    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1607,7 +1596,7 @@
       </c>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1">
+    <row r="13" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1631,7 +1620,7 @@
       </c>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" ht="15.75" thickBot="1">
+    <row r="14" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1655,7 +1644,7 @@
       </c>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="15.75" thickBot="1">
+    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1679,7 +1668,7 @@
       </c>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" ht="15.75" thickBot="1">
+    <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1703,7 +1692,7 @@
       </c>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1">
+    <row r="17" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1727,7 +1716,7 @@
       </c>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" ht="30.75" thickBot="1">
+    <row r="18" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1751,7 +1740,7 @@
       </c>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" ht="30.75" thickBot="1">
+    <row r="19" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1775,7 +1764,7 @@
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="30.75" thickBot="1">
+    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1799,7 +1788,7 @@
       </c>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" ht="30.75" thickBot="1">
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1823,7 +1812,7 @@
       </c>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8" ht="15.75" thickBot="1">
+    <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1847,7 +1836,7 @@
       </c>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" ht="15.75" thickBot="1">
+    <row r="23" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1871,7 +1860,7 @@
       </c>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" ht="15.75" thickBot="1">
+    <row r="24" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1895,7 +1884,7 @@
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" ht="30.75" thickBot="1">
+    <row r="25" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1919,7 +1908,7 @@
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" ht="15.75" thickBot="1">
+    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1943,17 +1932,17 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="63" spans="16:16">
+    <row r="63" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P63" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="64" spans="16:16">
+    <row r="64" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P64" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="65" spans="16:16">
+    <row r="65" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P65" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
Update project assignment file
</commit_message>
<xml_diff>
--- a/deadline_laptrinhmang.xlsx
+++ b/deadline_laptrinhmang.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GITHUB\UDM_05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA6817F-4768-4E4A-85FA-2D069DF3CE19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A771D5CC-ED69-4AF8-99B4-62DFD832974C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4996BFC1-5545-47D6-BEAA-54FAD06ABAD6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="84">
   <si>
     <t>STT</t>
   </si>
@@ -817,6 +817,21 @@
   </si>
   <si>
     <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>feature/multi-threading-server</t>
+  </si>
+  <si>
+    <t>feature/server-connection</t>
+  </si>
+  <si>
+    <t>Xây dựng GUI cấp quyền kết nối Client và tích hợp Logger vào Server để ghi nhận kết nối, thực thi lệnh và lỗi</t>
+  </si>
+  <si>
+    <t>GUI Server &amp; integrate logger</t>
+  </si>
+  <si>
+    <t>feature/server-gui</t>
   </si>
 </sst>
 </file>
@@ -1289,7 +1304,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0401913-6D54-40AB-B28F-C9358A79A9F4}">
-  <dimension ref="A1:P65"/>
+  <dimension ref="A1:P66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -1402,7 +1417,9 @@
       <c r="G4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
@@ -1546,7 +1563,9 @@
       <c r="G10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
@@ -1644,7 +1663,7 @@
       </c>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1666,7 +1685,9 @@
       <c r="G15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
@@ -1764,7 +1785,7 @@
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1772,13 +1793,13 @@
         <v>60</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F20" s="4">
         <v>46151</v>
@@ -1786,7 +1807,9 @@
       <c r="G20" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="H20" s="2"/>
+      <c r="H20" s="2" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
@@ -1796,13 +1819,13 @@
         <v>60</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F21" s="4">
         <v>46151</v>
@@ -1820,13 +1843,13 @@
         <v>60</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>30</v>
+        <v>64</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F22" s="4">
         <v>46151</v>
@@ -1844,13 +1867,13 @@
         <v>60</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F23" s="4">
         <v>46151</v>
@@ -1865,26 +1888,26 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F24" s="4">
-        <v>46365</v>
+        <v>46151</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>28</v>
       </c>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1892,13 +1915,13 @@
         <v>70</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F25" s="4">
         <v>46365</v>
@@ -1908,7 +1931,7 @@
       </c>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1916,13 +1939,13 @@
         <v>70</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="F26" s="4">
         <v>46365</v>
@@ -1932,24 +1955,48 @@
       </c>
       <c r="H26" s="2"/>
     </row>
-    <row r="63" spans="16:16" x14ac:dyDescent="0.3">
-      <c r="P63" t="s">
-        <v>78</v>
-      </c>
+    <row r="27" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="4">
+        <v>46365</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" s="2"/>
     </row>
     <row r="64" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P64" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
     </row>
     <row r="65" spans="16:16" x14ac:dyDescent="0.3">
       <c r="P65" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="66" spans="16:16" x14ac:dyDescent="0.3">
+      <c r="P66" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="G3:G26">
+  <conditionalFormatting sqref="G3:G27">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"IN PROGRESS"</formula>
     </cfRule>
@@ -1961,10 +2008,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G26" xr:uid="{C9A071F8-5EB0-444A-917D-D71EEB6D3E39}">
-      <formula1>$P$63:$P$65</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G27" xr:uid="{C9A071F8-5EB0-444A-917D-D71EEB6D3E39}">
+      <formula1>$P$64:$P$66</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>